<commit_message>
Armar el libro de KPIs con tres hojas y corregir las tablas que sí se leen.
Datos alimenta los SUMAR.SI y el dashboard. La estandarización, la sesión 17 y la hoja 3 de la propuesta quedan como en las capturas claras.

Co-authored-by: sebsotoosolis-ui <sebsotoosolis-ui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/documentos/Creacion y extraccion de contenido.xlsx
+++ b/documentos/Creacion y extraccion de contenido.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesión 17" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja1'!$A$3:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sesión 17'!$A$3:$H$23</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Sesión 17'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,7 +32,13 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="18"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -41,7 +48,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001F2933"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
@@ -50,18 +57,24 @@
       <color rgb="001B3A4B"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="005C6B7A"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B3A4B"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -78,8 +91,23 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF4EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF2FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -87,19 +115,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
     <border>
       <left style="thin">
-        <color rgb="00D5DEE7"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00D5DEE7"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00D5DEE7"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D5DEE7"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
@@ -109,41 +136,39 @@
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,23 +536,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="38" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Creación y extracción de contenido</t>
+          <t>SESIÓN 17 – CREACIÓN Y EXTRACCIÓN</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -538,59 +563,72 @@
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
     </row>
-    <row r="2" ht="10" customHeight="1"/>
-    <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>CONCATENAR()  y  EXTRAE()</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Apellido</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Nombre completo</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Prefijo</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>No. empleado</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="4" t="n">
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Juan</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Pérez</t>
         </is>
@@ -600,73 +638,69 @@
           <t>CV-2026-001</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Juan Pérez</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="9" t="n">
+      <c r="E4" s="8">
+        <f>CONCATENATE(B4," ",C4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="9">
+        <f>MID(D4,1,2)</f>
+        <v/>
+      </c>
+      <c r="G4" s="10">
+        <f>VALUE(MID(D4,4,4))</f>
+        <v/>
+      </c>
+      <c r="H4" s="9">
+        <f>MID(D4,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>María</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>López</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>CV-2026-002</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>María López</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="E5" s="8">
+        <f>CONCATENATE(B5," ",C5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="9">
+        <f>MID(D5,1,2)</f>
+        <v/>
+      </c>
+      <c r="G5" s="10">
+        <f>VALUE(MID(D5,4,4))</f>
+        <v/>
+      </c>
+      <c r="H5" s="9">
+        <f>MID(D5,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Carlos</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>García</t>
         </is>
@@ -676,73 +710,69 @@
           <t>CV-2026-003</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Carlos García</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="9" t="n">
+      <c r="E6" s="8">
+        <f>CONCATENATE(B6," ",C6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="9">
+        <f>MID(D6,1,2)</f>
+        <v/>
+      </c>
+      <c r="G6" s="10">
+        <f>VALUE(MID(D6,4,4))</f>
+        <v/>
+      </c>
+      <c r="H6" s="9">
+        <f>MID(D6,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Ana</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Martínez</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>CV-2026-004</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Ana Martínez</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="E7" s="8">
+        <f>CONCATENATE(B7," ",C7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="9">
+        <f>MID(D7,1,2)</f>
+        <v/>
+      </c>
+      <c r="G7" s="10">
+        <f>VALUE(MID(D7,4,4))</f>
+        <v/>
+      </c>
+      <c r="H7" s="9">
+        <f>MID(D7,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Pedro</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Ramos</t>
         </is>
@@ -752,73 +782,69 @@
           <t>CV-2026-005</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Pedro Ramos</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="9" t="n">
+      <c r="E8" s="8">
+        <f>CONCATENATE(B8," ",C8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="9">
+        <f>MID(D8,1,2)</f>
+        <v/>
+      </c>
+      <c r="G8" s="10">
+        <f>VALUE(MID(D8,4,4))</f>
+        <v/>
+      </c>
+      <c r="H8" s="9">
+        <f>MID(D8,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Sofía</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Hernández</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>CV-2026-006</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Sofía Hernández</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="E9" s="8">
+        <f>CONCATENATE(B9," ",C9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="9">
+        <f>MID(D9,1,2)</f>
+        <v/>
+      </c>
+      <c r="G9" s="10">
+        <f>VALUE(MID(D9,4,4))</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>MID(D9,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Diego</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Navarro</t>
         </is>
@@ -828,73 +854,69 @@
           <t>CV-2026-007</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Diego Navarro</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="9" t="n">
+      <c r="E10" s="8">
+        <f>CONCATENATE(B10," ",C10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="9">
+        <f>MID(D10,1,2)</f>
+        <v/>
+      </c>
+      <c r="G10" s="10">
+        <f>VALUE(MID(D10,4,4))</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>MID(D10,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Laura</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Morales</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>CV-2026-008</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Laura Morales</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="4" t="n">
+      <c r="E11" s="8">
+        <f>CONCATENATE(B11," ",C11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9">
+        <f>MID(D11,1,2)</f>
+        <v/>
+      </c>
+      <c r="G11" s="10">
+        <f>VALUE(MID(D11,4,4))</f>
+        <v/>
+      </c>
+      <c r="H11" s="9">
+        <f>MID(D11,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Jorge</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Torres</t>
         </is>
@@ -904,73 +926,69 @@
           <t>CV-2026-009</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Jorge Torres</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="n">
+      <c r="E12" s="8">
+        <f>CONCATENATE(B12," ",C12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="9">
+        <f>MID(D12,1,2)</f>
+        <v/>
+      </c>
+      <c r="G12" s="10">
+        <f>VALUE(MID(D12,4,4))</f>
+        <v/>
+      </c>
+      <c r="H12" s="9">
+        <f>MID(D12,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Fernanda</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Cruz</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>CV-2026-010</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>Fernanda Cruz</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="4" t="n">
+      <c r="E13" s="8">
+        <f>CONCATENATE(B13," ",C13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="9">
+        <f>MID(D13,1,2)</f>
+        <v/>
+      </c>
+      <c r="G13" s="10">
+        <f>VALUE(MID(D13,4,4))</f>
+        <v/>
+      </c>
+      <c r="H13" s="9">
+        <f>MID(D13,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Ricardo</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Silva</t>
         </is>
@@ -980,73 +998,69 @@
           <t>CV-2026-011</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Ricardo Silva</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="9" t="n">
+      <c r="E14" s="8">
+        <f>CONCATENATE(B14," ",C14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="9">
+        <f>MID(D14,1,2)</f>
+        <v/>
+      </c>
+      <c r="G14" s="10">
+        <f>VALUE(MID(D14,4,4))</f>
+        <v/>
+      </c>
+      <c r="H14" s="9">
+        <f>MID(D14,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Valeria</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>Mendoza</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>CV-2026-012</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>Valeria Mendoza</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="4" t="n">
+      <c r="E15" s="8">
+        <f>CONCATENATE(B15," ",C15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>MID(D15,1,2)</f>
+        <v/>
+      </c>
+      <c r="G15" s="10">
+        <f>VALUE(MID(D15,4,4))</f>
+        <v/>
+      </c>
+      <c r="H15" s="9">
+        <f>MID(D15,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Miguel</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Castro</t>
         </is>
@@ -1056,73 +1070,69 @@
           <t>CV-2026-013</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Miguel Castro</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="9" t="n">
+      <c r="E16" s="8">
+        <f>CONCATENATE(B16," ",C16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="9">
+        <f>MID(D16,1,2)</f>
+        <v/>
+      </c>
+      <c r="G16" s="10">
+        <f>VALUE(MID(D16,4,4))</f>
+        <v/>
+      </c>
+      <c r="H16" s="9">
+        <f>MID(D16,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Paola</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Romero</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>CV-2026-014</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>Paola Romero</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="4" t="n">
+      <c r="E17" s="8">
+        <f>CONCATENATE(B17," ",C17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="9">
+        <f>MID(D17,1,2)</f>
+        <v/>
+      </c>
+      <c r="G17" s="10">
+        <f>VALUE(MID(D17,4,4))</f>
+        <v/>
+      </c>
+      <c r="H17" s="9">
+        <f>MID(D17,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Andrés</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Vega</t>
         </is>
@@ -1132,73 +1142,69 @@
           <t>CV-2026-015</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Andrés Vega</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="9" t="n">
+      <c r="E18" s="8">
+        <f>CONCATENATE(B18," ",C18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="9">
+        <f>MID(D18,1,2)</f>
+        <v/>
+      </c>
+      <c r="G18" s="10">
+        <f>VALUE(MID(D18,4,4))</f>
+        <v/>
+      </c>
+      <c r="H18" s="9">
+        <f>MID(D18,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Elena</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Santos</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>CV-2026-016</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>Elena Santos</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G19" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="4" t="n">
+      <c r="E19" s="8">
+        <f>CONCATENATE(B19," ",C19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="9">
+        <f>MID(D19,1,2)</f>
+        <v/>
+      </c>
+      <c r="G19" s="10">
+        <f>VALUE(MID(D19,4,4))</f>
+        <v/>
+      </c>
+      <c r="H19" s="9">
+        <f>MID(D19,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Bruno</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Gómez</t>
         </is>
@@ -1208,73 +1214,69 @@
           <t>CV-2026-017</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Bruno Gómez</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="9" t="n">
+      <c r="E20" s="8">
+        <f>CONCATENATE(B20," ",C20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="9">
+        <f>MID(D20,1,2)</f>
+        <v/>
+      </c>
+      <c r="G20" s="10">
+        <f>VALUE(MID(D20,4,4))</f>
+        <v/>
+      </c>
+      <c r="H20" s="9">
+        <f>MID(D20,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Camila</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Ramírez</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>CV-2026-018</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
-        <is>
-          <t>Camila Ramírez</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="4" t="n">
+      <c r="E21" s="8">
+        <f>CONCATENATE(B21," ",C21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="9">
+        <f>MID(D21,1,2)</f>
+        <v/>
+      </c>
+      <c r="G21" s="10">
+        <f>VALUE(MID(D21,4,4))</f>
+        <v/>
+      </c>
+      <c r="H21" s="9">
+        <f>MID(D21,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Tomás</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Ortega</t>
         </is>
@@ -1284,69 +1286,74 @@
           <t>CV-2026-019</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>Tomás Ortega</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="9" t="n">
+      <c r="E22" s="8">
+        <f>CONCATENATE(B22," ",C22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="9">
+        <f>MID(D22,1,2)</f>
+        <v/>
+      </c>
+      <c r="G22" s="10">
+        <f>VALUE(MID(D22,4,4))</f>
+        <v/>
+      </c>
+      <c r="H22" s="9">
+        <f>MID(D22,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Natalia</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Flores</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>CV-2026-020</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>Natalia Flores</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>001</t>
+      <c r="E23" s="8">
+        <f>CONCATENATE(B23," ",C23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="9">
+        <f>MID(D23,1,2)</f>
+        <v/>
+      </c>
+      <c r="G23" s="10">
+        <f>VALUE(MID(D23,4,4))</f>
+        <v/>
+      </c>
+      <c r="H23" s="9">
+        <f>MID(D23,9,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Verde: CONCATENAR arma el nombre completo.  Azul: EXTRAE saca el prefijo (1,2), el año (4,4) y el número de empleado (9,3) desde el código.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:H23"/>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.45" right="0.45" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>